<commit_message>
Flag the rows Royal Wood Shop removed from the species sheet
The master list is built from the Products tab, which never saw the deletions
Brad made on the species tab — so all 62 codes he took out came back as
ordinary rows, and the archive-on-import check would find nothing removed.

They are shaded orange in the Code column now, with the reason in the header
note, so he can delete them again to confirm or leave them to keep the product.
Pink still means a code used by two products; the two sets do not overlap.

The v8/v9/v10 audit workbooks are gitignored — history, not inputs.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017k9FbEX1dxXBmE8gNPMCPT
</commit_message>
<xml_diff>
--- a/RoyalWoodShop_Master_Product_List_v1.xlsx
+++ b/RoyalWoodShop_Master_Product_List_v1.xlsx
@@ -48,7 +48,7 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Blank on 84 rows that have never had a product code — they cannot be imported until they do. Pink cells are codes used by two different products; one code has to mean one product.</t>
+          <t xml:space="preserve">Blank on 84 rows that have never had a product code — they cannot be imported until they do. PINK = this code is used by two different products; one code has to mean one product. ORANGE = you removed this row from the previous species sheet. It is back because this list is built from the full product record. Delete the row again to confirm, or leave it to keep the product.</t>
         </r>
       </text>
     </comment>
@@ -7730,7 +7730,7 @@
       <family val="2"/>
     </font>
   </fonts>
-  <fills count="6">
+  <fills count="7">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -7752,12 +7752,18 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFCE4E4"/>
-        <bgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFCE4D6"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
+        <bgColor rgb="FFFCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFCE4D6"/>
         <bgColor rgb="FFFCE4E4"/>
       </patternFill>
     </fill>
@@ -7811,7 +7817,7 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="8">
+  <cellXfs count="9">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
@@ -7844,6 +7850,10 @@
       <alignment horizontal="center" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
+    <xf numFmtId="164" fontId="5" fillId="6" borderId="1" xfId="0" applyFont="true" applyBorder="true" applyAlignment="false" applyProtection="false">
+      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
+      <protection locked="true" hidden="false"/>
+    </xf>
   </cellXfs>
   <cellStyles count="6">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -7853,7 +7863,7 @@
     <cellStyle name="Currency [0]" xfId="18" builtinId="7"/>
     <cellStyle name="Percent" xfId="19" builtinId="5"/>
   </cellStyles>
-  <dxfs count="6">
+  <dxfs count="7">
     <dxf>
       <fill>
         <patternFill patternType="solid">
@@ -7873,6 +7883,14 @@
       <fill>
         <patternFill patternType="solid">
           <fgColor rgb="FFFFFFFF"/>
+          <bgColor rgb="FF000000"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFCE4D6"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -7938,8 +7956,8 @@
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFCCFFCC"/>
       <rgbColor rgb="FFFCE4E4"/>
+      <rgbColor rgb="FFFCE4D6"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
@@ -8762,7 +8780,7 @@
       <c r="A12" s="3" t="s">
         <v>85</v>
       </c>
-      <c r="B12" s="3" t="s">
+      <c r="B12" s="8" t="s">
         <v>86</v>
       </c>
       <c r="C12" s="3" t="s">
@@ -10889,7 +10907,7 @@
       <c r="A55" s="3" t="s">
         <v>290</v>
       </c>
-      <c r="B55" s="3" t="s">
+      <c r="B55" s="8" t="s">
         <v>291</v>
       </c>
       <c r="C55" s="3" t="s">
@@ -11034,7 +11052,7 @@
       <c r="A58" s="3" t="s">
         <v>306</v>
       </c>
-      <c r="B58" s="3" t="s">
+      <c r="B58" s="8" t="s">
         <v>307</v>
       </c>
       <c r="C58" s="3" t="s">
@@ -11181,7 +11199,7 @@
       <c r="A61" s="3" t="s">
         <v>317</v>
       </c>
-      <c r="B61" s="3" t="s">
+      <c r="B61" s="8" t="s">
         <v>318</v>
       </c>
       <c r="C61" s="3" t="s">
@@ -11228,7 +11246,7 @@
       <c r="A62" s="3" t="s">
         <v>321</v>
       </c>
-      <c r="B62" s="3" t="s">
+      <c r="B62" s="8" t="s">
         <v>322</v>
       </c>
       <c r="C62" s="3" t="s">
@@ -11324,7 +11342,7 @@
       <c r="A64" s="3" t="s">
         <v>332</v>
       </c>
-      <c r="B64" s="3" t="s">
+      <c r="B64" s="8" t="s">
         <v>333</v>
       </c>
       <c r="C64" s="3" t="s">
@@ -11518,7 +11536,7 @@
       <c r="A68" s="3" t="s">
         <v>351</v>
       </c>
-      <c r="B68" s="3" t="s">
+      <c r="B68" s="8" t="s">
         <v>352</v>
       </c>
       <c r="C68" s="3" t="s">
@@ -12067,7 +12085,7 @@
       <c r="A79" s="3" t="s">
         <v>398</v>
       </c>
-      <c r="B79" s="3" t="s">
+      <c r="B79" s="8" t="s">
         <v>399</v>
       </c>
       <c r="C79" s="3" t="s">
@@ -12163,7 +12181,7 @@
       <c r="A81" s="3" t="s">
         <v>407</v>
       </c>
-      <c r="B81" s="3" t="s">
+      <c r="B81" s="8" t="s">
         <v>408</v>
       </c>
       <c r="C81" s="3" t="s">
@@ -12702,7 +12720,7 @@
       <c r="A92" s="3" t="s">
         <v>455</v>
       </c>
-      <c r="B92" s="3" t="s">
+      <c r="B92" s="8" t="s">
         <v>456</v>
       </c>
       <c r="C92" s="3" t="s">
@@ -13090,7 +13108,7 @@
       <c r="A100" s="3" t="s">
         <v>493</v>
       </c>
-      <c r="B100" s="3" t="s">
+      <c r="B100" s="8" t="s">
         <v>494</v>
       </c>
       <c r="C100" s="3" t="s">
@@ -13845,7 +13863,7 @@
       <c r="A115" s="3" t="s">
         <v>563</v>
       </c>
-      <c r="B115" s="3" t="s">
+      <c r="B115" s="8" t="s">
         <v>564</v>
       </c>
       <c r="C115" s="3" t="s">
@@ -13943,7 +13961,7 @@
       <c r="A117" s="3" t="s">
         <v>573</v>
       </c>
-      <c r="B117" s="3" t="s">
+      <c r="B117" s="8" t="s">
         <v>574</v>
       </c>
       <c r="C117" s="3" t="s">
@@ -14527,7 +14545,7 @@
       <c r="A129" s="3" t="s">
         <v>631</v>
       </c>
-      <c r="B129" s="3" t="s">
+      <c r="B129" s="8" t="s">
         <v>632</v>
       </c>
       <c r="C129" s="3" t="s">
@@ -14821,7 +14839,7 @@
       <c r="A135" s="3" t="s">
         <v>655</v>
       </c>
-      <c r="B135" s="3" t="s">
+      <c r="B135" s="8" t="s">
         <v>656</v>
       </c>
       <c r="C135" s="3" t="s">
@@ -15017,7 +15035,7 @@
       <c r="A139" s="3" t="s">
         <v>673</v>
       </c>
-      <c r="B139" s="3" t="s">
+      <c r="B139" s="8" t="s">
         <v>674</v>
       </c>
       <c r="C139" s="3" t="s">
@@ -15113,7 +15131,7 @@
       <c r="A141" s="3" t="s">
         <v>680</v>
       </c>
-      <c r="B141" s="3" t="s">
+      <c r="B141" s="8" t="s">
         <v>681</v>
       </c>
       <c r="C141" s="3" t="s">
@@ -15160,7 +15178,7 @@
       <c r="A142" s="3" t="s">
         <v>684</v>
       </c>
-      <c r="B142" s="3" t="s">
+      <c r="B142" s="8" t="s">
         <v>685</v>
       </c>
       <c r="C142" s="3" t="s">
@@ -15307,7 +15325,7 @@
       <c r="A145" s="3" t="s">
         <v>699</v>
       </c>
-      <c r="B145" s="3" t="s">
+      <c r="B145" s="8" t="s">
         <v>700</v>
       </c>
       <c r="C145" s="3" t="s">
@@ -15354,7 +15372,7 @@
       <c r="A146" s="3" t="s">
         <v>703</v>
       </c>
-      <c r="B146" s="3" t="s">
+      <c r="B146" s="8" t="s">
         <v>704</v>
       </c>
       <c r="C146" s="3" t="s">
@@ -15552,7 +15570,7 @@
       <c r="A150" s="3" t="s">
         <v>717</v>
       </c>
-      <c r="B150" s="3" t="s">
+      <c r="B150" s="8" t="s">
         <v>718</v>
       </c>
       <c r="C150" s="3" t="s">
@@ -16109,7 +16127,7 @@
       <c r="A161" s="3" t="s">
         <v>766</v>
       </c>
-      <c r="B161" s="3" t="s">
+      <c r="B161" s="8" t="s">
         <v>767</v>
       </c>
       <c r="C161" s="3" t="s">
@@ -16454,7 +16472,7 @@
       <c r="A168" s="3" t="s">
         <v>796</v>
       </c>
-      <c r="B168" s="3" t="s">
+      <c r="B168" s="8" t="s">
         <v>797</v>
       </c>
       <c r="C168" s="3" t="s">
@@ -16501,7 +16519,7 @@
       <c r="A169" s="3" t="s">
         <v>801</v>
       </c>
-      <c r="B169" s="3" t="s">
+      <c r="B169" s="8" t="s">
         <v>802</v>
       </c>
       <c r="C169" s="3" t="s">
@@ -16548,7 +16566,7 @@
       <c r="A170" s="3" t="s">
         <v>806</v>
       </c>
-      <c r="B170" s="3" t="s">
+      <c r="B170" s="8" t="s">
         <v>807</v>
       </c>
       <c r="C170" s="3" t="s">
@@ -17291,7 +17309,7 @@
       <c r="A185" s="3" t="s">
         <v>869</v>
       </c>
-      <c r="B185" s="3" t="s">
+      <c r="B185" s="8" t="s">
         <v>870</v>
       </c>
       <c r="C185" s="3" t="s">
@@ -17338,7 +17356,7 @@
       <c r="A186" s="3" t="s">
         <v>873</v>
       </c>
-      <c r="B186" s="3" t="s">
+      <c r="B186" s="8" t="s">
         <v>874</v>
       </c>
       <c r="C186" s="3" t="s">
@@ -17640,7 +17658,7 @@
       <c r="A192" s="3" t="s">
         <v>896</v>
       </c>
-      <c r="B192" s="3" t="s">
+      <c r="B192" s="8" t="s">
         <v>897</v>
       </c>
       <c r="C192" s="3" t="s">
@@ -17736,7 +17754,7 @@
       <c r="A194" s="3" t="s">
         <v>904</v>
       </c>
-      <c r="B194" s="3" t="s">
+      <c r="B194" s="8" t="s">
         <v>905</v>
       </c>
       <c r="C194" s="3" t="s">
@@ -17830,7 +17848,7 @@
       <c r="A196" s="3" t="s">
         <v>912</v>
       </c>
-      <c r="B196" s="3" t="s">
+      <c r="B196" s="8" t="s">
         <v>913</v>
       </c>
       <c r="C196" s="3" t="s">
@@ -18673,7 +18691,7 @@
       <c r="A213" s="3" t="s">
         <v>973</v>
       </c>
-      <c r="B213" s="3" t="s">
+      <c r="B213" s="8" t="s">
         <v>974</v>
       </c>
       <c r="C213" s="3" t="s">
@@ -19459,7 +19477,7 @@
       <c r="A229" s="3" t="s">
         <v>1045</v>
       </c>
-      <c r="B229" s="3" t="s">
+      <c r="B229" s="8" t="s">
         <v>1046</v>
       </c>
       <c r="C229" s="3" t="s">
@@ -19555,7 +19573,7 @@
       <c r="A231" s="3" t="s">
         <v>1054</v>
       </c>
-      <c r="B231" s="3" t="s">
+      <c r="B231" s="8" t="s">
         <v>1055</v>
       </c>
       <c r="C231" s="3" t="s">
@@ -27708,7 +27726,7 @@
       <c r="A406" s="3" t="s">
         <v>1572</v>
       </c>
-      <c r="B406" s="3" t="s">
+      <c r="B406" s="8" t="s">
         <v>1573</v>
       </c>
       <c r="C406" s="3" t="s">
@@ -27847,7 +27865,7 @@
       <c r="A409" s="3" t="s">
         <v>1587</v>
       </c>
-      <c r="B409" s="3" t="s">
+      <c r="B409" s="8" t="s">
         <v>1588</v>
       </c>
       <c r="C409" s="3" t="s">
@@ -28172,7 +28190,7 @@
       <c r="A416" s="3" t="s">
         <v>1612</v>
       </c>
-      <c r="B416" s="3" t="s">
+      <c r="B416" s="8" t="s">
         <v>1613</v>
       </c>
       <c r="C416" s="3" t="s">
@@ -29927,7 +29945,7 @@
       <c r="A455" s="3" t="s">
         <v>1779</v>
       </c>
-      <c r="B455" s="3" t="s">
+      <c r="B455" s="8" t="s">
         <v>1780</v>
       </c>
       <c r="C455" s="3" t="s">
@@ -30144,7 +30162,7 @@
       <c r="A460" s="3" t="s">
         <v>1799</v>
       </c>
-      <c r="B460" s="3" t="s">
+      <c r="B460" s="8" t="s">
         <v>1800</v>
       </c>
       <c r="C460" s="3" t="s">
@@ -30412,7 +30430,7 @@
       <c r="A466" s="3" t="s">
         <v>1819</v>
       </c>
-      <c r="B466" s="3" t="s">
+      <c r="B466" s="8" t="s">
         <v>1820</v>
       </c>
       <c r="C466" s="3" t="s">
@@ -30455,7 +30473,7 @@
       <c r="A467" s="3" t="s">
         <v>1823</v>
       </c>
-      <c r="B467" s="3" t="s">
+      <c r="B467" s="8" t="s">
         <v>1824</v>
       </c>
       <c r="C467" s="3" t="s">
@@ -30856,7 +30874,7 @@
       <c r="A476" s="3" t="s">
         <v>1858</v>
       </c>
-      <c r="B476" s="3" t="s">
+      <c r="B476" s="8" t="s">
         <v>1859</v>
       </c>
       <c r="C476" s="3" t="s">
@@ -30899,7 +30917,7 @@
       <c r="A477" s="3" t="s">
         <v>1861</v>
       </c>
-      <c r="B477" s="3" t="s">
+      <c r="B477" s="8" t="s">
         <v>1862</v>
       </c>
       <c r="C477" s="3" t="s">
@@ -31179,7 +31197,7 @@
       <c r="A483" s="3" t="s">
         <v>1887</v>
       </c>
-      <c r="B483" s="3" t="s">
+      <c r="B483" s="8" t="s">
         <v>1888</v>
       </c>
       <c r="C483" s="3" t="s">
@@ -31365,7 +31383,7 @@
       <c r="A487" s="3" t="s">
         <v>1904</v>
       </c>
-      <c r="B487" s="3" t="s">
+      <c r="B487" s="8" t="s">
         <v>1905</v>
       </c>
       <c r="C487" s="3" t="s">
@@ -32284,7 +32302,7 @@
       <c r="A508" s="3" t="s">
         <v>1965</v>
       </c>
-      <c r="B508" s="3" t="s">
+      <c r="B508" s="8" t="s">
         <v>1966</v>
       </c>
       <c r="C508" s="3" t="s">
@@ -32329,7 +32347,7 @@
       <c r="A509" s="3" t="s">
         <v>1969</v>
       </c>
-      <c r="B509" s="3" t="s">
+      <c r="B509" s="8" t="s">
         <v>1970</v>
       </c>
       <c r="C509" s="3" t="s">
@@ -32421,7 +32439,7 @@
       <c r="A511" s="3" t="s">
         <v>1977</v>
       </c>
-      <c r="B511" s="3" t="s">
+      <c r="B511" s="8" t="s">
         <v>1978</v>
       </c>
       <c r="C511" s="3" t="s">
@@ -32466,7 +32484,7 @@
       <c r="A512" s="3" t="s">
         <v>1981</v>
       </c>
-      <c r="B512" s="3" t="s">
+      <c r="B512" s="8" t="s">
         <v>1982</v>
       </c>
       <c r="C512" s="3" t="s">
@@ -32556,7 +32574,7 @@
       <c r="A514" s="3" t="s">
         <v>1987</v>
       </c>
-      <c r="B514" s="3" t="s">
+      <c r="B514" s="8" t="s">
         <v>1988</v>
       </c>
       <c r="C514" s="3" t="s">
@@ -32601,7 +32619,7 @@
       <c r="A515" s="3" t="s">
         <v>1991</v>
       </c>
-      <c r="B515" s="3" t="s">
+      <c r="B515" s="8" t="s">
         <v>1992</v>
       </c>
       <c r="C515" s="3" t="s">
@@ -32693,7 +32711,7 @@
       <c r="A517" s="3" t="s">
         <v>1999</v>
       </c>
-      <c r="B517" s="3" t="s">
+      <c r="B517" s="8" t="s">
         <v>2000</v>
       </c>
       <c r="C517" s="3" t="s">
@@ -32738,7 +32756,7 @@
       <c r="A518" s="3" t="s">
         <v>2003</v>
       </c>
-      <c r="B518" s="3" t="s">
+      <c r="B518" s="8" t="s">
         <v>2004</v>
       </c>
       <c r="C518" s="3" t="s">
@@ -32783,7 +32801,7 @@
       <c r="A519" s="3" t="s">
         <v>2007</v>
       </c>
-      <c r="B519" s="3" t="s">
+      <c r="B519" s="8" t="s">
         <v>2008</v>
       </c>
       <c r="C519" s="3" t="s">
@@ -43884,7 +43902,7 @@
     </row>
     <row r="786" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A786" s="3"/>
-      <c r="B786" s="3" t="s">
+      <c r="B786" s="8" t="s">
         <v>2426</v>
       </c>
       <c r="C786" s="5"/>
@@ -43925,7 +43943,7 @@
     </row>
     <row r="787" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A787" s="3"/>
-      <c r="B787" s="3" t="s">
+      <c r="B787" s="8" t="s">
         <v>2427</v>
       </c>
       <c r="C787" s="5"/>
@@ -43966,7 +43984,7 @@
     </row>
     <row r="788" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A788" s="3"/>
-      <c r="B788" s="3" t="s">
+      <c r="B788" s="8" t="s">
         <v>2428</v>
       </c>
       <c r="C788" s="5"/>
@@ -44007,7 +44025,7 @@
     </row>
     <row r="789" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A789" s="3"/>
-      <c r="B789" s="3" t="s">
+      <c r="B789" s="8" t="s">
         <v>2429</v>
       </c>
       <c r="C789" s="5"/>
@@ -44048,7 +44066,7 @@
     </row>
     <row r="790" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A790" s="3"/>
-      <c r="B790" s="3" t="s">
+      <c r="B790" s="8" t="s">
         <v>2430</v>
       </c>
       <c r="C790" s="5"/>
@@ -44089,7 +44107,7 @@
     </row>
     <row r="791" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A791" s="3"/>
-      <c r="B791" s="3" t="s">
+      <c r="B791" s="8" t="s">
         <v>2431</v>
       </c>
       <c r="C791" s="5"/>
@@ -44130,7 +44148,7 @@
     </row>
     <row r="792" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A792" s="3"/>
-      <c r="B792" s="3" t="s">
+      <c r="B792" s="8" t="s">
         <v>2432</v>
       </c>
       <c r="C792" s="5"/>
@@ -46458,7 +46476,7 @@
     </row>
     <row r="846" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A846" s="3"/>
-      <c r="B846" s="3" t="s">
+      <c r="B846" s="8" t="s">
         <v>2495</v>
       </c>
       <c r="C846" s="5"/>
@@ -47039,7 +47057,7 @@
     </row>
     <row r="859" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A859" s="3"/>
-      <c r="B859" s="3" t="s">
+      <c r="B859" s="8" t="s">
         <v>2512</v>
       </c>
       <c r="C859" s="5"/>

</xml_diff>

<commit_message>
Make the two Code flags tell themselves apart
They were FFFCE4E4 and FFFCE4D6 — fourteen points apart on the blue channel and
identical on screen, with the only explanation buried in a header comment. Two
different meanings looked like one.

Salmon now means a duplicated code and something to fix; blue means the row was
deleted from the previous species sheet and is back for a decision. Every shaded
cell carries its own note, so hovering it says which it is and what to do.

Co-Authored-By: Claude Opus 5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_017k9FbEX1dxXBmE8gNPMCPT
</commit_message>
<xml_diff>
--- a/RoyalWoodShop_Master_Product_List_v1.xlsx
+++ b/RoyalWoodShop_Master_Product_List_v1.xlsx
@@ -48,7 +48,962 @@
             <rFont val="Arial"/>
             <family val="2"/>
           </rPr>
-          <t xml:space="preserve">Blank on 84 rows that have never had a product code — they cannot be imported until they do. PINK = this code is used by two different products; one code has to mean one product. ORANGE = you removed this row from the previous species sheet. It is back because this list is built from the full product record. Delete the row again to confirm, or leave it to keep the product.</t>
+          <t xml:space="preserve">Blank on 84 rows that have never had a product code — they cannot be imported until they do.
+SALMON = this code is used by two different products. Something to fix.
+BLUE = you removed this row from the previous species sheet. For information.
+Hover any shaded cell and it tells you which it is and what to do.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B2" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">SALMON — this product code is on two rows for two different products.
+The import matches on code, so it cannot tell them apart: only the first row is imported and the second product gets nothing.
+Fix it by giving one of them its own code, or by deleting one row if they are the same product recorded twice.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B12" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B55" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B58" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B61" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B62" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B64" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B68" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B79" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B81" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B92" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B100" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B115" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B117" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B129" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B135" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B139" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B141" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B142" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B145" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B146" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B150" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B161" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B168" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B169" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B170" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B185" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B186" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B192" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B194" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B196" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B197" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">SALMON — this product code is on two rows for two different products.
+The import matches on code, so it cannot tell them apart: only the first row is imported and the second product gets nothing.
+Fix it by giving one of them its own code, or by deleting one row if they are the same product recorded twice.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B213" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B229" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B231" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B406" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B409" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B416" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B425" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">SALMON — this product code is on two rows for two different products.
+The import matches on code, so it cannot tell them apart: only the first row is imported and the second product gets nothing.
+Fix it by giving one of them its own code, or by deleting one row if they are the same product recorded twice.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B426" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">SALMON — this product code is on two rows for two different products.
+The import matches on code, so it cannot tell them apart: only the first row is imported and the second product gets nothing.
+Fix it by giving one of them its own code, or by deleting one row if they are the same product recorded twice.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B455" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B460" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B462" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">SALMON — this product code is on two rows for two different products.
+The import matches on code, so it cannot tell them apart: only the first row is imported and the second product gets nothing.
+Fix it by giving one of them its own code, or by deleting one row if they are the same product recorded twice.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B463" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">SALMON — this product code is on two rows for two different products.
+The import matches on code, so it cannot tell them apart: only the first row is imported and the second product gets nothing.
+Fix it by giving one of them its own code, or by deleting one row if they are the same product recorded twice.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B466" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B467" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B476" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B477" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B483" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B487" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B508" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B509" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B511" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B512" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B514" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B515" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B517" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B518" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B519" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B786" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B787" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B788" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B789" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B790" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B791" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B792" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B846" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="B859" authorId="0">
+      <text>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <rFont val="Arial"/>
+            <family val="2"/>
+          </rPr>
+          <t xml:space="preserve">BLUE — you deleted this row from the previous species sheet.
+It is back because this list is built from the full product record, which never saw that deletion. Nothing is wrong with the row.
+Delete it again if the product is discontinued, or leave it to keep the product.</t>
         </r>
       </text>
     </comment>
@@ -7746,25 +8701,25 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFF7C7AC"/>
-        <bgColor rgb="FFD9D9D9"/>
+        <bgColor rgb="FFF8CBAD"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFCE4E4"/>
-        <bgColor rgb="FFFCE4D6"/>
+        <fgColor rgb="FFF8CBAD"/>
+        <bgColor rgb="FFF7C7AC"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFFF2CC"/>
-        <bgColor rgb="FFFCE4D6"/>
+        <bgColor rgb="FFFFFFFF"/>
       </patternFill>
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="FFFCE4D6"/>
-        <bgColor rgb="FFFCE4E4"/>
+        <fgColor rgb="FFDDEBF7"/>
+        <bgColor rgb="FFD9D9D9"/>
       </patternFill>
     </fill>
   </fills>
@@ -7890,7 +8845,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFCE4D6"/>
+          <fgColor rgb="FFDDEBF7"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -7898,7 +8853,7 @@
     <dxf>
       <fill>
         <patternFill patternType="solid">
-          <fgColor rgb="FFFCE4E4"/>
+          <fgColor rgb="FFF8CBAD"/>
           <bgColor rgb="FF000000"/>
         </patternFill>
       </fill>
@@ -7936,12 +8891,12 @@
       <rgbColor rgb="FF808000"/>
       <rgbColor rgb="FF800080"/>
       <rgbColor rgb="FF008080"/>
-      <rgbColor rgb="FFC0C0C0"/>
+      <rgbColor rgb="FFF7C7AC"/>
       <rgbColor rgb="FF808080"/>
       <rgbColor rgb="FF9999FF"/>
       <rgbColor rgb="FF993366"/>
       <rgbColor rgb="FFFFF2CC"/>
-      <rgbColor rgb="FFCCFFFF"/>
+      <rgbColor rgb="FFDDEBF7"/>
       <rgbColor rgb="FF660066"/>
       <rgbColor rgb="FFFF8080"/>
       <rgbColor rgb="FF0066CC"/>
@@ -7956,12 +8911,12 @@
       <rgbColor rgb="FF0000FF"/>
       <rgbColor rgb="FF00CCFF"/>
       <rgbColor rgb="FFCCFFFF"/>
-      <rgbColor rgb="FFFCE4E4"/>
-      <rgbColor rgb="FFFCE4D6"/>
+      <rgbColor rgb="FFCCFFCC"/>
+      <rgbColor rgb="FFFFFF99"/>
       <rgbColor rgb="FF99CCFF"/>
       <rgbColor rgb="FFFF99CC"/>
       <rgbColor rgb="FFCC99FF"/>
-      <rgbColor rgb="FFF7C7AC"/>
+      <rgbColor rgb="FFF8CBAD"/>
       <rgbColor rgb="FF3366FF"/>
       <rgbColor rgb="FF33CCCC"/>
       <rgbColor rgb="FF99CC00"/>

</xml_diff>